<commit_message>
Fill remaining FSX dual stock_sector from listing-keyed official sources.
Copy GICS from official TMX/CSE leftover matches, ASX listed-companies plus
ISIN.xls, Nasdaq Nordic shares, JPX 33-industry including the Information
and Communication label variant, SET NSIN/search, Euronext ICB, LJSE NACE,
Nasdaq Baltic, Aquis, Spotlight, and multi-token non-OTC primary same-issuer
or US/CA CUSIP listings. Skip OTC, one-token issuer keys, XETRA/German
same-ticker ISIN-change, unmapped CSE Life Sciences/CleanTech, JPX Others,
and scanner/EODHD/FinanceDatabase fills. Core FSX Stock missing sectors
646→258. Does not claim 99%. Stacks on core-trust-identity-fills.
</commit_message>
<xml_diff>
--- a/data/nasdaq_baltic_verification/shares.xlsx
+++ b/data/nasdaq_baltic_verification/shares.xlsx
@@ -1209,13 +1209,13 @@
         <v>25</v>
       </c>
       <c r="G2">
-        <v>1.79333333</v>
+        <v>1.82</v>
       </c>
       <c r="H2">
         <v>1.8</v>
       </c>
       <c r="I2">
-        <v>1.82</v>
+        <v>1.83</v>
       </c>
       <c r="J2">
         <v>1.76</v>
@@ -1224,22 +1224,25 @@
         <v>1.82</v>
       </c>
       <c r="L2">
-        <v>1.82</v>
+        <v>1.83</v>
+      </c>
+      <c r="M2">
+        <v>0.55</v>
       </c>
       <c r="N2">
         <v>1.76</v>
       </c>
       <c r="O2">
-        <v>1.81</v>
+        <v>1.83</v>
       </c>
       <c r="P2">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="Q2">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="R2">
-        <v>5.38</v>
+        <v>41.86</v>
       </c>
       <c r="S2" t="s">
         <v>26</v>
@@ -1392,7 +1395,7 @@
         <v>32</v>
       </c>
       <c r="G5">
-        <v>3.84457939</v>
+        <v>3.84450608</v>
       </c>
       <c r="H5">
         <v>3.85</v>
@@ -1407,22 +1410,25 @@
         <v>3.85</v>
       </c>
       <c r="L5">
-        <v>3.85</v>
+        <v>3.84</v>
+      </c>
+      <c r="M5">
+        <v>-0.26</v>
       </c>
       <c r="N5">
         <v>3.84</v>
       </c>
       <c r="O5">
-        <v>3.85</v>
+        <v>3.84</v>
       </c>
       <c r="P5">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="Q5">
-        <v>4125</v>
+        <v>4525</v>
       </c>
       <c r="R5">
-        <v>15858.89</v>
+        <v>17396.39</v>
       </c>
       <c r="S5" t="s">
         <v>43</v>
@@ -1513,7 +1519,7 @@
         <v>38</v>
       </c>
       <c r="G7">
-        <v>0.08512414</v>
+        <v>0.08509359</v>
       </c>
       <c r="H7">
         <v>0.085</v>
@@ -1522,31 +1528,28 @@
         <v>0.0878</v>
       </c>
       <c r="J7">
-        <v>0.0842</v>
+        <v>0.0838</v>
       </c>
       <c r="K7">
         <v>0.085</v>
       </c>
       <c r="L7">
-        <v>0.0842</v>
-      </c>
-      <c r="M7">
-        <v>-0.94</v>
+        <v>0.085</v>
       </c>
       <c r="N7">
-        <v>0.0842</v>
+        <v>0.085</v>
       </c>
       <c r="O7">
         <v>0.085</v>
       </c>
       <c r="P7">
-        <v>349</v>
+        <v>370</v>
       </c>
       <c r="Q7">
-        <v>53623</v>
+        <v>55380</v>
       </c>
       <c r="R7">
-        <v>4564.612</v>
+        <v>4712.483</v>
       </c>
       <c r="S7" t="s">
         <v>33</v>
@@ -1575,7 +1578,7 @@
         <v>38</v>
       </c>
       <c r="G8">
-        <v>1.26965818</v>
+        <v>1.26891858</v>
       </c>
       <c r="H8">
         <v>1.27</v>
@@ -1584,31 +1587,31 @@
         <v>1.305</v>
       </c>
       <c r="J8">
-        <v>1.26</v>
+        <v>1.255</v>
       </c>
       <c r="K8">
         <v>1.275</v>
       </c>
       <c r="L8">
-        <v>1.27</v>
+        <v>1.255</v>
       </c>
       <c r="M8">
-        <v>-0.39</v>
+        <v>-1.57</v>
       </c>
       <c r="N8">
         <v>1.26</v>
       </c>
       <c r="O8">
-        <v>1.275</v>
+        <v>1.27</v>
       </c>
       <c r="P8">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="Q8">
-        <v>746</v>
+        <v>786</v>
       </c>
       <c r="R8">
-        <v>947.165</v>
+        <v>997.37</v>
       </c>
       <c r="S8" t="s">
         <v>33</v>
@@ -1699,7 +1702,7 @@
         <v>32</v>
       </c>
       <c r="G10">
-        <v>2.32815256</v>
+        <v>2.32819927</v>
       </c>
       <c r="H10">
         <v>2.34</v>
@@ -1720,19 +1723,19 @@
         <v>-0.43</v>
       </c>
       <c r="N10">
-        <v>2.325</v>
+        <v>2.33</v>
       </c>
       <c r="O10">
-        <v>2.33</v>
+        <v>2.335</v>
       </c>
       <c r="P10">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="Q10">
-        <v>30185</v>
+        <v>30893</v>
       </c>
       <c r="R10">
-        <v>70275.285</v>
+        <v>71925.06</v>
       </c>
       <c r="S10" t="s">
         <v>63</v>
@@ -1802,7 +1805,7 @@
         <v>32</v>
       </c>
       <c r="G12">
-        <v>1.6709477</v>
+        <v>1.67140037</v>
       </c>
       <c r="H12">
         <v>1.65</v>
@@ -1823,19 +1826,19 @@
         <v>2.13</v>
       </c>
       <c r="N12">
-        <v>1.67</v>
+        <v>1.675</v>
       </c>
       <c r="O12">
         <v>1.675</v>
       </c>
       <c r="P12">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="Q12">
-        <v>19236</v>
+        <v>20259</v>
       </c>
       <c r="R12">
-        <v>32142.35</v>
+        <v>33860.9</v>
       </c>
       <c r="S12" t="s">
         <v>63</v>
@@ -1864,7 +1867,7 @@
         <v>32</v>
       </c>
       <c r="G13">
-        <v>19.50839552</v>
+        <v>19.49725331</v>
       </c>
       <c r="H13">
         <v>19.5</v>
@@ -1873,28 +1876,31 @@
         <v>19.55</v>
       </c>
       <c r="J13">
-        <v>19.45</v>
+        <v>19.4</v>
       </c>
       <c r="K13">
         <v>19.5</v>
       </c>
       <c r="L13">
-        <v>19.5</v>
+        <v>19.4</v>
+      </c>
+      <c r="M13">
+        <v>-0.51</v>
       </c>
       <c r="N13">
-        <v>19.45</v>
+        <v>19.4</v>
       </c>
       <c r="O13">
         <v>19.5</v>
       </c>
       <c r="P13">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="Q13">
-        <v>804</v>
+        <v>983</v>
       </c>
       <c r="R13">
-        <v>15684.75</v>
+        <v>19165.8</v>
       </c>
       <c r="S13" t="s">
         <v>63</v>
@@ -1923,7 +1929,7 @@
         <v>25</v>
       </c>
       <c r="G14">
-        <v>6.75136986</v>
+        <v>6.75202703</v>
       </c>
       <c r="H14">
         <v>6.75</v>
@@ -1938,10 +1944,10 @@
         <v>6.7</v>
       </c>
       <c r="L14">
-        <v>6.75</v>
+        <v>6.8</v>
       </c>
       <c r="M14">
-        <v>0.75</v>
+        <v>1.49</v>
       </c>
       <c r="N14">
         <v>6.7</v>
@@ -1950,13 +1956,13 @@
         <v>6.8</v>
       </c>
       <c r="P14">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q14">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="R14">
-        <v>1971.4</v>
+        <v>1998.6</v>
       </c>
       <c r="S14" t="s">
         <v>33</v>
@@ -2076,7 +2082,7 @@
         <v>25</v>
       </c>
       <c r="G17">
-        <v>11.04245283</v>
+        <v>11.02836879</v>
       </c>
       <c r="H17">
         <v>11.2</v>
@@ -2085,31 +2091,31 @@
         <v>11.3</v>
       </c>
       <c r="J17">
-        <v>11.0</v>
+        <v>10.9</v>
       </c>
       <c r="K17">
         <v>11.2</v>
       </c>
       <c r="L17">
-        <v>11.0</v>
+        <v>10.9</v>
       </c>
       <c r="M17">
-        <v>-1.79</v>
+        <v>-2.68</v>
       </c>
       <c r="N17">
         <v>10.9</v>
       </c>
       <c r="O17">
-        <v>11.0</v>
+        <v>10.9</v>
       </c>
       <c r="P17">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="Q17">
-        <v>106</v>
+        <v>141</v>
       </c>
       <c r="R17">
-        <v>1170.5</v>
+        <v>1555.0</v>
       </c>
       <c r="S17" t="s">
         <v>26</v>
@@ -2185,7 +2191,7 @@
         <v>30.0</v>
       </c>
       <c r="N19">
-        <v>0.032</v>
+        <v>0.034</v>
       </c>
       <c r="O19">
         <v>0.039</v>
@@ -2226,7 +2232,7 @@
         <v>32</v>
       </c>
       <c r="G20">
-        <v>1.01965205</v>
+        <v>1.01976436</v>
       </c>
       <c r="H20">
         <v>1.02</v>
@@ -2250,13 +2256,13 @@
         <v>1.02</v>
       </c>
       <c r="P20">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="Q20">
-        <v>1049</v>
+        <v>1549</v>
       </c>
       <c r="R20">
-        <v>1069.615</v>
+        <v>1579.615</v>
       </c>
       <c r="S20" t="s">
         <v>97</v>
@@ -2285,7 +2291,7 @@
         <v>32</v>
       </c>
       <c r="G21">
-        <v>5.18373816</v>
+        <v>5.18366554</v>
       </c>
       <c r="H21">
         <v>5.2</v>
@@ -2309,16 +2315,16 @@
         <v>5.16</v>
       </c>
       <c r="O21">
-        <v>5.18</v>
+        <v>5.2</v>
       </c>
       <c r="P21">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="Q21">
-        <v>1161</v>
+        <v>1184</v>
       </c>
       <c r="R21">
-        <v>6018.32</v>
+        <v>6137.46</v>
       </c>
       <c r="S21" t="s">
         <v>26</v>
@@ -2347,7 +2353,7 @@
         <v>32</v>
       </c>
       <c r="G22">
-        <v>4.43792453</v>
+        <v>4.4387037</v>
       </c>
       <c r="H22">
         <v>4.49</v>
@@ -2362,22 +2368,25 @@
         <v>4.49</v>
       </c>
       <c r="L22">
-        <v>4.49</v>
+        <v>4.48</v>
+      </c>
+      <c r="M22">
+        <v>-0.22</v>
       </c>
       <c r="N22">
         <v>4.45</v>
       </c>
       <c r="O22">
-        <v>4.48</v>
+        <v>4.49</v>
       </c>
       <c r="P22">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q22">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R22">
-        <v>235.21</v>
+        <v>239.69</v>
       </c>
       <c r="S22" t="s">
         <v>48</v>
@@ -2406,7 +2415,7 @@
         <v>32</v>
       </c>
       <c r="G23">
-        <v>9.83996115</v>
+        <v>9.85407324</v>
       </c>
       <c r="H23">
         <v>9.74</v>
@@ -2421,25 +2430,25 @@
         <v>9.72</v>
       </c>
       <c r="L23">
-        <v>9.88</v>
+        <v>9.9</v>
       </c>
       <c r="M23">
-        <v>1.65</v>
+        <v>1.85</v>
       </c>
       <c r="N23">
-        <v>9.86</v>
+        <v>9.92</v>
       </c>
       <c r="O23">
-        <v>9.88</v>
+        <v>9.96</v>
       </c>
       <c r="P23">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="Q23">
-        <v>2574</v>
+        <v>3550</v>
       </c>
       <c r="R23">
-        <v>25328.06</v>
+        <v>34981.96</v>
       </c>
       <c r="S23" t="s">
         <v>63</v>
@@ -2468,7 +2477,7 @@
         <v>32</v>
       </c>
       <c r="G24">
-        <v>21.77170331</v>
+        <v>21.76905795</v>
       </c>
       <c r="H24">
         <v>21.85</v>
@@ -2495,13 +2504,13 @@
         <v>21.75</v>
       </c>
       <c r="P24">
-        <v>368</v>
+        <v>402</v>
       </c>
       <c r="Q24">
-        <v>22151</v>
+        <v>24659</v>
       </c>
       <c r="R24">
-        <v>482265.0</v>
+        <v>536803.2</v>
       </c>
       <c r="S24" t="s">
         <v>111</v>
@@ -2651,7 +2660,7 @@
         <v>32</v>
       </c>
       <c r="G27">
-        <v>63.71641086</v>
+        <v>63.69817792</v>
       </c>
       <c r="H27">
         <v>63.8</v>
@@ -2678,13 +2687,13 @@
         <v>63.6</v>
       </c>
       <c r="P27">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="Q27">
-        <v>847</v>
+        <v>933</v>
       </c>
       <c r="R27">
-        <v>53967.8</v>
+        <v>59430.4</v>
       </c>
       <c r="S27" t="s">
         <v>63</v>
@@ -2840,13 +2849,13 @@
         <v>27.0</v>
       </c>
       <c r="P30">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q30">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="R30">
-        <v>2484.0</v>
+        <v>2511.0</v>
       </c>
       <c r="S30" t="s">
         <v>63</v>
@@ -2875,13 +2884,13 @@
         <v>25</v>
       </c>
       <c r="G31">
-        <v>12.1</v>
+        <v>12.10882353</v>
       </c>
       <c r="H31">
         <v>12.1</v>
       </c>
       <c r="I31">
-        <v>12.1</v>
+        <v>12.2</v>
       </c>
       <c r="J31">
         <v>12.1</v>
@@ -2890,7 +2899,10 @@
         <v>12.1</v>
       </c>
       <c r="L31">
-        <v>12.1</v>
+        <v>12.2</v>
+      </c>
+      <c r="M31">
+        <v>0.83</v>
       </c>
       <c r="N31">
         <v>12.1</v>
@@ -2899,13 +2911,13 @@
         <v>12.2</v>
       </c>
       <c r="P31">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q31">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="R31">
-        <v>1125.3</v>
+        <v>1235.1</v>
       </c>
       <c r="S31" t="s">
         <v>33</v>
@@ -2934,7 +2946,7 @@
         <v>32</v>
       </c>
       <c r="G32">
-        <v>0.48434724</v>
+        <v>0.48435317</v>
       </c>
       <c r="H32">
         <v>0.484</v>
@@ -2955,19 +2967,19 @@
         <v>0.21</v>
       </c>
       <c r="N32">
-        <v>0.484</v>
+        <v>0.485</v>
       </c>
       <c r="O32">
         <v>0.485</v>
       </c>
       <c r="P32">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="Q32">
-        <v>11557</v>
+        <v>11663</v>
       </c>
       <c r="R32">
-        <v>5597.601</v>
+        <v>5649.011</v>
       </c>
       <c r="S32" t="s">
         <v>26</v>
@@ -2996,7 +3008,7 @@
         <v>38</v>
       </c>
       <c r="G33">
-        <v>2.11112882</v>
+        <v>2.11162907</v>
       </c>
       <c r="H33">
         <v>2.1</v>
@@ -3020,16 +3032,16 @@
         <v>2.06</v>
       </c>
       <c r="O33">
-        <v>2.12</v>
+        <v>2.14</v>
       </c>
       <c r="P33">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q33">
-        <v>1506</v>
+        <v>1596</v>
       </c>
       <c r="R33">
-        <v>3179.36</v>
+        <v>3370.16</v>
       </c>
       <c r="S33" t="s">
         <v>111</v>
@@ -3058,7 +3070,7 @@
         <v>38</v>
       </c>
       <c r="G34">
-        <v>1.14065164</v>
+        <v>1.13956083</v>
       </c>
       <c r="H34">
         <v>1.14</v>
@@ -3067,13 +3079,16 @@
         <v>1.15</v>
       </c>
       <c r="J34">
-        <v>1.14</v>
+        <v>1.135</v>
       </c>
       <c r="K34">
         <v>1.14</v>
       </c>
       <c r="L34">
-        <v>1.14</v>
+        <v>1.135</v>
+      </c>
+      <c r="M34">
+        <v>-0.44</v>
       </c>
       <c r="N34">
         <v>1.135</v>
@@ -3082,13 +3097,13 @@
         <v>1.14</v>
       </c>
       <c r="P34">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q34">
-        <v>2839</v>
+        <v>3518</v>
       </c>
       <c r="R34">
-        <v>3238.31</v>
+        <v>4008.975</v>
       </c>
       <c r="S34" t="s">
         <v>111</v>
@@ -3117,7 +3132,7 @@
         <v>32</v>
       </c>
       <c r="G35">
-        <v>3.26966551</v>
+        <v>3.2696642</v>
       </c>
       <c r="H35">
         <v>3.27</v>
@@ -3135,19 +3150,19 @@
         <v>3.27</v>
       </c>
       <c r="N35">
-        <v>3.265</v>
+        <v>3.27</v>
       </c>
       <c r="O35">
         <v>3.27</v>
       </c>
       <c r="P35">
-        <v>273</v>
+        <v>294</v>
       </c>
       <c r="Q35">
-        <v>47640</v>
+        <v>50834</v>
       </c>
       <c r="R35">
-        <v>155766.865</v>
+        <v>166210.11</v>
       </c>
       <c r="S35" t="s">
         <v>63</v>
@@ -3241,7 +3256,7 @@
         <v>3.42</v>
       </c>
       <c r="O37">
-        <v>3.47</v>
+        <v>3.46</v>
       </c>
       <c r="P37">
         <v>14</v>
@@ -3279,7 +3294,7 @@
         <v>25</v>
       </c>
       <c r="G38">
-        <v>2.1532078</v>
+        <v>2.15452269</v>
       </c>
       <c r="H38">
         <v>2.12</v>
@@ -3294,25 +3309,25 @@
         <v>2.09</v>
       </c>
       <c r="L38">
-        <v>2.19</v>
+        <v>2.15</v>
       </c>
       <c r="M38">
-        <v>4.78</v>
+        <v>2.87</v>
       </c>
       <c r="N38">
-        <v>2.16</v>
+        <v>2.12</v>
       </c>
       <c r="O38">
-        <v>2.18</v>
+        <v>2.17</v>
       </c>
       <c r="P38">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="Q38">
-        <v>1487</v>
+        <v>1917</v>
       </c>
       <c r="R38">
-        <v>3201.82</v>
+        <v>4130.22</v>
       </c>
       <c r="S38" t="s">
         <v>154</v>
@@ -3368,13 +3383,13 @@
         <v>10.45</v>
       </c>
       <c r="P39">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q39">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="R39">
-        <v>20.8</v>
+        <v>1060.8</v>
       </c>
       <c r="S39" t="s">
         <v>43</v>
@@ -3403,7 +3418,7 @@
         <v>25</v>
       </c>
       <c r="G40">
-        <v>5.08697118</v>
+        <v>5.09087373</v>
       </c>
       <c r="H40">
         <v>5.3</v>
@@ -3418,25 +3433,25 @@
         <v>5.3</v>
       </c>
       <c r="L40">
-        <v>5.0</v>
+        <v>5.25</v>
       </c>
       <c r="M40">
-        <v>-5.66</v>
+        <v>-0.94</v>
       </c>
       <c r="N40">
-        <v>5.0</v>
+        <v>5.05</v>
       </c>
       <c r="O40">
-        <v>5.25</v>
+        <v>5.2</v>
       </c>
       <c r="P40">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="Q40">
-        <v>1631</v>
+        <v>1671</v>
       </c>
       <c r="R40">
-        <v>8296.85</v>
+        <v>8506.85</v>
       </c>
       <c r="S40" t="s">
         <v>162</v>
@@ -3527,7 +3542,7 @@
         <v>32</v>
       </c>
       <c r="G42">
-        <v>27.0799812</v>
+        <v>27.07996875</v>
       </c>
       <c r="H42">
         <v>27.15</v>
@@ -3554,13 +3569,13 @@
         <v>27.1</v>
       </c>
       <c r="P42">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="Q42">
-        <v>1596</v>
+        <v>1600</v>
       </c>
       <c r="R42">
-        <v>43219.65</v>
+        <v>43327.95</v>
       </c>
       <c r="S42" t="s">
         <v>26</v>
@@ -3589,7 +3604,7 @@
         <v>32</v>
       </c>
       <c r="G43">
-        <v>0.55765644</v>
+        <v>0.55770891</v>
       </c>
       <c r="H43">
         <v>0.56</v>
@@ -3604,10 +3619,7 @@
         <v>0.56</v>
       </c>
       <c r="L43">
-        <v>0.556</v>
-      </c>
-      <c r="M43">
-        <v>-0.71</v>
+        <v>0.56</v>
       </c>
       <c r="N43">
         <v>0.556</v>
@@ -3616,13 +3628,13 @@
         <v>0.56</v>
       </c>
       <c r="P43">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q43">
-        <v>2183</v>
+        <v>2233</v>
       </c>
       <c r="R43">
-        <v>1217.364</v>
+        <v>1245.364</v>
       </c>
       <c r="S43" t="s">
         <v>26</v>
@@ -3716,7 +3728,7 @@
         <v>0.75</v>
       </c>
       <c r="O45">
-        <v>0.76</v>
+        <v>0.758</v>
       </c>
       <c r="P45">
         <v>9</v>
@@ -3816,7 +3828,7 @@
         <v>25</v>
       </c>
       <c r="G47">
-        <v>0.03724681</v>
+        <v>0.0348915</v>
       </c>
       <c r="H47">
         <v>0.039</v>
@@ -3831,25 +3843,25 @@
         <v>0.03</v>
       </c>
       <c r="L47">
-        <v>0.038</v>
+        <v>0.031</v>
       </c>
       <c r="M47">
-        <v>26.67</v>
+        <v>3.33</v>
       </c>
       <c r="N47">
-        <v>0.031</v>
+        <v>0.03</v>
       </c>
       <c r="O47">
         <v>0.038</v>
       </c>
       <c r="P47">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q47">
-        <v>1487</v>
+        <v>2387</v>
       </c>
       <c r="R47">
-        <v>55.386</v>
+        <v>83.286</v>
       </c>
       <c r="S47" t="s">
         <v>162</v>
@@ -3878,7 +3890,7 @@
         <v>38</v>
       </c>
       <c r="G48">
-        <v>0.05498936</v>
+        <v>0.05492262</v>
       </c>
       <c r="H48">
         <v>0.0538</v>
@@ -3893,25 +3905,25 @@
         <v>0.054</v>
       </c>
       <c r="L48">
-        <v>0.055</v>
+        <v>0.0548</v>
       </c>
       <c r="M48">
-        <v>1.85</v>
+        <v>1.48</v>
       </c>
       <c r="N48">
         <v>0.054</v>
       </c>
       <c r="O48">
-        <v>0.055</v>
+        <v>0.0548</v>
       </c>
       <c r="P48">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q48">
-        <v>1128</v>
+        <v>1742</v>
       </c>
       <c r="R48">
-        <v>62.028</v>
+        <v>95.6752</v>
       </c>
       <c r="S48" t="s">
         <v>33</v>
@@ -3975,7 +3987,7 @@
         <v>32</v>
       </c>
       <c r="G50">
-        <v>1.80693753</v>
+        <v>1.80693339</v>
       </c>
       <c r="H50">
         <v>1.81</v>
@@ -3990,22 +4002,25 @@
         <v>1.81</v>
       </c>
       <c r="L50">
-        <v>1.81</v>
+        <v>1.805</v>
+      </c>
+      <c r="M50">
+        <v>-0.28</v>
       </c>
       <c r="N50">
-        <v>1.805</v>
+        <v>1.8</v>
       </c>
       <c r="O50">
         <v>1.81</v>
       </c>
       <c r="P50">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="Q50">
-        <v>2449</v>
+        <v>2462</v>
       </c>
       <c r="R50">
-        <v>4425.19</v>
+        <v>4448.67</v>
       </c>
       <c r="S50" t="s">
         <v>33</v>
@@ -4034,7 +4049,7 @@
         <v>38</v>
       </c>
       <c r="G51">
-        <v>0.33</v>
+        <v>0.30092308</v>
       </c>
       <c r="H51">
         <v>0.33</v>
@@ -4043,31 +4058,31 @@
         <v>0.33</v>
       </c>
       <c r="J51">
-        <v>0.33</v>
+        <v>0.294</v>
       </c>
       <c r="K51">
         <v>0.32</v>
       </c>
       <c r="L51">
-        <v>0.33</v>
+        <v>0.294</v>
       </c>
       <c r="M51">
-        <v>3.13</v>
+        <v>-8.13</v>
       </c>
       <c r="N51">
         <v>0.292</v>
       </c>
       <c r="O51">
-        <v>0.33</v>
+        <v>0.328</v>
       </c>
       <c r="P51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q51">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="R51">
-        <v>1.65</v>
+        <v>7.824</v>
       </c>
       <c r="S51" t="s">
         <v>26</v>
@@ -4096,7 +4111,7 @@
         <v>32</v>
       </c>
       <c r="G52">
-        <v>0.89654925</v>
+        <v>0.89632286</v>
       </c>
       <c r="H52">
         <v>0.9</v>
@@ -4105,31 +4120,31 @@
         <v>0.9</v>
       </c>
       <c r="J52">
-        <v>0.895</v>
+        <v>0.894</v>
       </c>
       <c r="K52">
         <v>0.9</v>
       </c>
       <c r="L52">
-        <v>0.896</v>
+        <v>0.894</v>
       </c>
       <c r="M52">
-        <v>-0.44</v>
+        <v>-0.67</v>
       </c>
       <c r="N52">
         <v>0.894</v>
       </c>
       <c r="O52">
-        <v>0.896</v>
+        <v>0.894</v>
       </c>
       <c r="P52">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="Q52">
-        <v>107255</v>
+        <v>122187</v>
       </c>
       <c r="R52">
-        <v>96159.39</v>
+        <v>109519.001</v>
       </c>
     </row>
     <row r="53" spans="1:20">
@@ -4152,7 +4167,7 @@
         <v>32</v>
       </c>
       <c r="G53">
-        <v>4.45593909</v>
+        <v>4.4731934</v>
       </c>
       <c r="H53">
         <v>4.54</v>
@@ -4167,7 +4182,10 @@
         <v>4.5</v>
       </c>
       <c r="L53">
-        <v>4.5</v>
+        <v>4.48</v>
+      </c>
+      <c r="M53">
+        <v>-0.44</v>
       </c>
       <c r="N53">
         <v>4.46</v>
@@ -4176,13 +4194,13 @@
         <v>4.52</v>
       </c>
       <c r="P53">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="Q53">
-        <v>788</v>
+        <v>2668</v>
       </c>
       <c r="R53">
-        <v>3511.28</v>
+        <v>11934.48</v>
       </c>
       <c r="S53" t="s">
         <v>33</v>
@@ -4211,7 +4229,7 @@
         <v>32</v>
       </c>
       <c r="G54">
-        <v>16.43611111</v>
+        <v>16.44252137</v>
       </c>
       <c r="H54">
         <v>16.5</v>
@@ -4226,25 +4244,25 @@
         <v>16.6</v>
       </c>
       <c r="L54">
-        <v>16.4</v>
+        <v>16.5</v>
       </c>
       <c r="M54">
-        <v>-1.2</v>
+        <v>-0.6</v>
       </c>
       <c r="N54">
-        <v>16.4</v>
+        <v>16.5</v>
       </c>
       <c r="O54">
-        <v>16.45</v>
+        <v>16.5</v>
       </c>
       <c r="P54">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="Q54">
-        <v>54</v>
+        <v>234</v>
       </c>
       <c r="R54">
-        <v>887.55</v>
+        <v>3847.55</v>
       </c>
       <c r="S54" t="s">
         <v>154</v>
@@ -4376,7 +4394,7 @@
         <v>32</v>
       </c>
       <c r="G57">
-        <v>1.07257792</v>
+        <v>1.07216533</v>
       </c>
       <c r="H57">
         <v>1.075</v>
@@ -4391,25 +4409,25 @@
         <v>1.08</v>
       </c>
       <c r="L57">
-        <v>1.06</v>
+        <v>1.065</v>
       </c>
       <c r="M57">
-        <v>-1.85</v>
+        <v>-1.39</v>
       </c>
       <c r="N57">
         <v>1.06</v>
       </c>
       <c r="O57">
-        <v>1.08</v>
+        <v>1.075</v>
       </c>
       <c r="P57">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q57">
-        <v>1893</v>
+        <v>2002</v>
       </c>
       <c r="R57">
-        <v>2030.39</v>
+        <v>2146.475</v>
       </c>
       <c r="S57" t="s">
         <v>43</v>
@@ -4500,7 +4518,7 @@
         <v>32</v>
       </c>
       <c r="G59">
-        <v>0.64593359</v>
+        <v>0.64594582</v>
       </c>
       <c r="H59">
         <v>0.647</v>
@@ -4515,25 +4533,22 @@
         <v>0.646</v>
       </c>
       <c r="L59">
-        <v>0.647</v>
-      </c>
-      <c r="M59">
-        <v>0.15</v>
+        <v>0.646</v>
       </c>
       <c r="N59">
         <v>0.646</v>
       </c>
       <c r="O59">
-        <v>0.647</v>
+        <v>0.646</v>
       </c>
       <c r="P59">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="Q59">
-        <v>115420</v>
+        <v>129893</v>
       </c>
       <c r="R59">
-        <v>74553.655</v>
+        <v>83903.841</v>
       </c>
       <c r="S59" t="s">
         <v>43</v>
@@ -4562,7 +4577,7 @@
         <v>32</v>
       </c>
       <c r="G60">
-        <v>2.2314222</v>
+        <v>2.23209208</v>
       </c>
       <c r="H60">
         <v>2.23</v>
@@ -4589,13 +4604,13 @@
         <v>2.24</v>
       </c>
       <c r="P60">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="Q60">
-        <v>28934</v>
+        <v>31385</v>
       </c>
       <c r="R60">
-        <v>64563.97</v>
+        <v>70054.21</v>
       </c>
       <c r="S60" t="s">
         <v>154</v>
@@ -4624,7 +4639,7 @@
         <v>32</v>
       </c>
       <c r="G61">
-        <v>9.02400323</v>
+        <v>9.01369341</v>
       </c>
       <c r="H61">
         <v>9.05</v>
@@ -4645,19 +4660,19 @@
         <v>-0.44</v>
       </c>
       <c r="N61">
-        <v>9.0</v>
+        <v>9.01</v>
       </c>
       <c r="O61">
         <v>9.01</v>
       </c>
       <c r="P61">
-        <v>282</v>
+        <v>404</v>
       </c>
       <c r="Q61">
-        <v>6190</v>
+        <v>10979</v>
       </c>
       <c r="R61">
-        <v>55858.58</v>
+        <v>98961.34</v>
       </c>
       <c r="S61" t="s">
         <v>43</v>
@@ -4727,7 +4742,7 @@
         <v>32</v>
       </c>
       <c r="G63">
-        <v>1.21106577</v>
+        <v>1.21113757</v>
       </c>
       <c r="H63">
         <v>1.208</v>
@@ -4751,16 +4766,16 @@
         <v>1.21</v>
       </c>
       <c r="O63">
-        <v>1.212</v>
+        <v>1.214</v>
       </c>
       <c r="P63">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="Q63">
-        <v>17683</v>
+        <v>18696</v>
       </c>
       <c r="R63">
-        <v>21415.276</v>
+        <v>22643.428</v>
       </c>
       <c r="S63" t="s">
         <v>26</v>
@@ -4789,7 +4804,7 @@
         <v>32</v>
       </c>
       <c r="G64">
-        <v>10.88387609</v>
+        <v>10.87583128</v>
       </c>
       <c r="H64">
         <v>10.85</v>
@@ -4813,13 +4828,13 @@
         <v>10.85</v>
       </c>
       <c r="P64">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="Q64">
-        <v>1259</v>
+        <v>1624</v>
       </c>
       <c r="R64">
-        <v>13702.8</v>
+        <v>17662.35</v>
       </c>
       <c r="S64" t="s">
         <v>111</v>
@@ -4848,7 +4863,7 @@
         <v>38</v>
       </c>
       <c r="G65">
-        <v>0.33606832</v>
+        <v>0.32764706</v>
       </c>
       <c r="H65">
         <v>0.34</v>
@@ -4857,31 +4872,31 @@
         <v>0.34</v>
       </c>
       <c r="J65">
-        <v>0.334</v>
+        <v>0.32</v>
       </c>
       <c r="K65">
         <v>0.34</v>
       </c>
       <c r="L65">
-        <v>0.334</v>
+        <v>0.32</v>
       </c>
       <c r="M65">
-        <v>-1.76</v>
+        <v>-5.88</v>
       </c>
       <c r="N65">
-        <v>0.334</v>
+        <v>0.32</v>
       </c>
       <c r="O65">
         <v>0.34</v>
       </c>
       <c r="P65">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="Q65">
-        <v>322</v>
+        <v>850</v>
       </c>
       <c r="R65">
-        <v>108.214</v>
+        <v>278.5</v>
       </c>
       <c r="S65" t="s">
         <v>43</v>
@@ -4910,7 +4925,7 @@
         <v>38</v>
       </c>
       <c r="G66">
-        <v>9.87631579</v>
+        <v>9.85</v>
       </c>
       <c r="H66">
         <v>9.85</v>
@@ -4919,13 +4934,16 @@
         <v>9.9</v>
       </c>
       <c r="J66">
-        <v>9.85</v>
+        <v>9.6</v>
       </c>
       <c r="K66">
         <v>9.9</v>
       </c>
       <c r="L66">
-        <v>9.9</v>
+        <v>9.6</v>
+      </c>
+      <c r="M66">
+        <v>-3.03</v>
       </c>
       <c r="N66">
         <v>9.6</v>
@@ -4934,13 +4952,13 @@
         <v>9.9</v>
       </c>
       <c r="P66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q66">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="R66">
-        <v>187.65</v>
+        <v>206.85</v>
       </c>
       <c r="S66" t="s">
         <v>43</v>
@@ -4969,7 +4987,7 @@
         <v>25</v>
       </c>
       <c r="G67">
-        <v>4.41469127</v>
+        <v>4.41570577</v>
       </c>
       <c r="H67">
         <v>4.43</v>
@@ -4993,13 +5011,13 @@
         <v>4.43</v>
       </c>
       <c r="P67">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q67">
-        <v>1409</v>
+        <v>1509</v>
       </c>
       <c r="R67">
-        <v>6220.3</v>
+        <v>6663.3</v>
       </c>
       <c r="S67" t="s">
         <v>43</v>
@@ -5028,7 +5046,7 @@
         <v>32</v>
       </c>
       <c r="G68">
-        <v>15.30085586</v>
+        <v>15.30082322</v>
       </c>
       <c r="H68">
         <v>15.3</v>
@@ -5055,13 +5073,13 @@
         <v>15.3</v>
       </c>
       <c r="P68">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="Q68">
-        <v>1110</v>
+        <v>1154</v>
       </c>
       <c r="R68">
-        <v>16983.95</v>
+        <v>17657.15</v>
       </c>
       <c r="S68" t="s">
         <v>33</v>
@@ -5090,13 +5108,13 @@
         <v>38</v>
       </c>
       <c r="G69">
-        <v>2.9433126</v>
+        <v>2.94375191</v>
       </c>
       <c r="H69">
         <v>2.94</v>
       </c>
       <c r="I69">
-        <v>2.96</v>
+        <v>2.98</v>
       </c>
       <c r="J69">
         <v>2.9</v>
@@ -5105,10 +5123,10 @@
         <v>2.94</v>
       </c>
       <c r="L69">
-        <v>2.96</v>
+        <v>2.98</v>
       </c>
       <c r="M69">
-        <v>0.68</v>
+        <v>1.36</v>
       </c>
       <c r="N69">
         <v>2.94</v>
@@ -5117,13 +5135,13 @@
         <v>2.98</v>
       </c>
       <c r="P69">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="Q69">
-        <v>1286</v>
+        <v>1306</v>
       </c>
       <c r="R69">
-        <v>3785.1</v>
+        <v>3844.54</v>
       </c>
       <c r="S69" t="s">
         <v>33</v>
@@ -5238,13 +5256,13 @@
         <v>25</v>
       </c>
       <c r="G2">
-        <v>1.79333333</v>
+        <v>1.82</v>
       </c>
       <c r="H2">
         <v>1.8</v>
       </c>
       <c r="I2">
-        <v>1.82</v>
+        <v>1.83</v>
       </c>
       <c r="J2">
         <v>1.76</v>
@@ -5253,22 +5271,25 @@
         <v>1.82</v>
       </c>
       <c r="L2">
-        <v>1.82</v>
+        <v>1.83</v>
+      </c>
+      <c r="M2">
+        <v>0.55</v>
       </c>
       <c r="N2">
         <v>1.76</v>
       </c>
       <c r="O2">
-        <v>1.81</v>
+        <v>1.83</v>
       </c>
       <c r="P2">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="Q2">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="R2">
-        <v>5.38</v>
+        <v>41.86</v>
       </c>
       <c r="S2" t="s">
         <v>26</v>
@@ -5421,7 +5442,7 @@
         <v>32</v>
       </c>
       <c r="G5">
-        <v>2.32815256</v>
+        <v>2.32819927</v>
       </c>
       <c r="H5">
         <v>2.34</v>
@@ -5442,19 +5463,19 @@
         <v>-0.43</v>
       </c>
       <c r="N5">
-        <v>2.325</v>
+        <v>2.33</v>
       </c>
       <c r="O5">
-        <v>2.33</v>
+        <v>2.335</v>
       </c>
       <c r="P5">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="Q5">
-        <v>30185</v>
+        <v>30893</v>
       </c>
       <c r="R5">
-        <v>70275.285</v>
+        <v>71925.06</v>
       </c>
       <c r="S5" t="s">
         <v>63</v>
@@ -5483,7 +5504,7 @@
         <v>32</v>
       </c>
       <c r="G6">
-        <v>19.50839552</v>
+        <v>19.49725331</v>
       </c>
       <c r="H6">
         <v>19.5</v>
@@ -5492,28 +5513,31 @@
         <v>19.55</v>
       </c>
       <c r="J6">
-        <v>19.45</v>
+        <v>19.4</v>
       </c>
       <c r="K6">
         <v>19.5</v>
       </c>
       <c r="L6">
-        <v>19.5</v>
+        <v>19.4</v>
+      </c>
+      <c r="M6">
+        <v>-0.51</v>
       </c>
       <c r="N6">
-        <v>19.45</v>
+        <v>19.4</v>
       </c>
       <c r="O6">
         <v>19.5</v>
       </c>
       <c r="P6">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="Q6">
-        <v>804</v>
+        <v>983</v>
       </c>
       <c r="R6">
-        <v>15684.75</v>
+        <v>19165.8</v>
       </c>
       <c r="S6" t="s">
         <v>63</v>
@@ -5592,7 +5616,7 @@
         <v>30.0</v>
       </c>
       <c r="N8">
-        <v>0.032</v>
+        <v>0.034</v>
       </c>
       <c r="O8">
         <v>0.039</v>
@@ -5633,7 +5657,7 @@
         <v>32</v>
       </c>
       <c r="G9">
-        <v>5.18373816</v>
+        <v>5.18366554</v>
       </c>
       <c r="H9">
         <v>5.2</v>
@@ -5657,16 +5681,16 @@
         <v>5.16</v>
       </c>
       <c r="O9">
-        <v>5.18</v>
+        <v>5.2</v>
       </c>
       <c r="P9">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="Q9">
-        <v>1161</v>
+        <v>1184</v>
       </c>
       <c r="R9">
-        <v>6018.32</v>
+        <v>6137.46</v>
       </c>
       <c r="S9" t="s">
         <v>26</v>
@@ -5695,7 +5719,7 @@
         <v>32</v>
       </c>
       <c r="G10">
-        <v>4.43792453</v>
+        <v>4.4387037</v>
       </c>
       <c r="H10">
         <v>4.49</v>
@@ -5710,22 +5734,25 @@
         <v>4.49</v>
       </c>
       <c r="L10">
-        <v>4.49</v>
+        <v>4.48</v>
+      </c>
+      <c r="M10">
+        <v>-0.22</v>
       </c>
       <c r="N10">
         <v>4.45</v>
       </c>
       <c r="O10">
-        <v>4.48</v>
+        <v>4.49</v>
       </c>
       <c r="P10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q10">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R10">
-        <v>235.21</v>
+        <v>239.69</v>
       </c>
       <c r="S10" t="s">
         <v>48</v>
@@ -5754,7 +5781,7 @@
         <v>32</v>
       </c>
       <c r="G11">
-        <v>63.71641086</v>
+        <v>63.69817792</v>
       </c>
       <c r="H11">
         <v>63.8</v>
@@ -5781,13 +5808,13 @@
         <v>63.6</v>
       </c>
       <c r="P11">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="Q11">
-        <v>847</v>
+        <v>933</v>
       </c>
       <c r="R11">
-        <v>53967.8</v>
+        <v>59430.4</v>
       </c>
       <c r="S11" t="s">
         <v>63</v>
@@ -5816,7 +5843,7 @@
         <v>32</v>
       </c>
       <c r="G12">
-        <v>3.26966551</v>
+        <v>3.2696642</v>
       </c>
       <c r="H12">
         <v>3.27</v>
@@ -5834,19 +5861,19 @@
         <v>3.27</v>
       </c>
       <c r="N12">
-        <v>3.265</v>
+        <v>3.27</v>
       </c>
       <c r="O12">
         <v>3.27</v>
       </c>
       <c r="P12">
-        <v>273</v>
+        <v>294</v>
       </c>
       <c r="Q12">
-        <v>47640</v>
+        <v>50834</v>
       </c>
       <c r="R12">
-        <v>155766.865</v>
+        <v>166210.11</v>
       </c>
       <c r="S12" t="s">
         <v>63</v>
@@ -5940,7 +5967,7 @@
         <v>3.42</v>
       </c>
       <c r="O14">
-        <v>3.47</v>
+        <v>3.46</v>
       </c>
       <c r="P14">
         <v>14</v>
@@ -5978,7 +6005,7 @@
         <v>25</v>
       </c>
       <c r="G15">
-        <v>2.1532078</v>
+        <v>2.15452269</v>
       </c>
       <c r="H15">
         <v>2.12</v>
@@ -5993,25 +6020,25 @@
         <v>2.09</v>
       </c>
       <c r="L15">
-        <v>2.19</v>
+        <v>2.15</v>
       </c>
       <c r="M15">
-        <v>4.78</v>
+        <v>2.87</v>
       </c>
       <c r="N15">
-        <v>2.16</v>
+        <v>2.12</v>
       </c>
       <c r="O15">
-        <v>2.18</v>
+        <v>2.17</v>
       </c>
       <c r="P15">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="Q15">
-        <v>1487</v>
+        <v>1917</v>
       </c>
       <c r="R15">
-        <v>3201.82</v>
+        <v>4130.22</v>
       </c>
       <c r="S15" t="s">
         <v>154</v>
@@ -6040,7 +6067,7 @@
         <v>25</v>
       </c>
       <c r="G16">
-        <v>5.08697118</v>
+        <v>5.09087373</v>
       </c>
       <c r="H16">
         <v>5.3</v>
@@ -6055,25 +6082,25 @@
         <v>5.3</v>
       </c>
       <c r="L16">
-        <v>5.0</v>
+        <v>5.25</v>
       </c>
       <c r="M16">
-        <v>-5.66</v>
+        <v>-0.94</v>
       </c>
       <c r="N16">
-        <v>5.0</v>
+        <v>5.05</v>
       </c>
       <c r="O16">
-        <v>5.25</v>
+        <v>5.2</v>
       </c>
       <c r="P16">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="Q16">
-        <v>1631</v>
+        <v>1671</v>
       </c>
       <c r="R16">
-        <v>8296.85</v>
+        <v>8506.85</v>
       </c>
       <c r="S16" t="s">
         <v>162</v>
@@ -6164,7 +6191,7 @@
         <v>32</v>
       </c>
       <c r="G18">
-        <v>27.0799812</v>
+        <v>27.07996875</v>
       </c>
       <c r="H18">
         <v>27.15</v>
@@ -6191,13 +6218,13 @@
         <v>27.1</v>
       </c>
       <c r="P18">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="Q18">
-        <v>1596</v>
+        <v>1600</v>
       </c>
       <c r="R18">
-        <v>43219.65</v>
+        <v>43327.95</v>
       </c>
       <c r="S18" t="s">
         <v>26</v>
@@ -6226,7 +6253,7 @@
         <v>32</v>
       </c>
       <c r="G19">
-        <v>0.55765644</v>
+        <v>0.55770891</v>
       </c>
       <c r="H19">
         <v>0.56</v>
@@ -6241,10 +6268,7 @@
         <v>0.56</v>
       </c>
       <c r="L19">
-        <v>0.556</v>
-      </c>
-      <c r="M19">
-        <v>-0.71</v>
+        <v>0.56</v>
       </c>
       <c r="N19">
         <v>0.556</v>
@@ -6253,13 +6277,13 @@
         <v>0.56</v>
       </c>
       <c r="P19">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q19">
-        <v>2183</v>
+        <v>2233</v>
       </c>
       <c r="R19">
-        <v>1217.364</v>
+        <v>1245.364</v>
       </c>
       <c r="S19" t="s">
         <v>26</v>
@@ -6350,7 +6374,7 @@
         <v>25</v>
       </c>
       <c r="G21">
-        <v>0.03724681</v>
+        <v>0.0348915</v>
       </c>
       <c r="H21">
         <v>0.039</v>
@@ -6365,25 +6389,25 @@
         <v>0.03</v>
       </c>
       <c r="L21">
-        <v>0.038</v>
+        <v>0.031</v>
       </c>
       <c r="M21">
-        <v>26.67</v>
+        <v>3.33</v>
       </c>
       <c r="N21">
-        <v>0.031</v>
+        <v>0.03</v>
       </c>
       <c r="O21">
         <v>0.038</v>
       </c>
       <c r="P21">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q21">
-        <v>1487</v>
+        <v>2387</v>
       </c>
       <c r="R21">
-        <v>55.386</v>
+        <v>83.286</v>
       </c>
       <c r="S21" t="s">
         <v>162</v>
@@ -6412,7 +6436,7 @@
         <v>38</v>
       </c>
       <c r="G22">
-        <v>0.05498936</v>
+        <v>0.05492262</v>
       </c>
       <c r="H22">
         <v>0.0538</v>
@@ -6427,25 +6451,25 @@
         <v>0.054</v>
       </c>
       <c r="L22">
-        <v>0.055</v>
+        <v>0.0548</v>
       </c>
       <c r="M22">
-        <v>1.85</v>
+        <v>1.48</v>
       </c>
       <c r="N22">
         <v>0.054</v>
       </c>
       <c r="O22">
-        <v>0.055</v>
+        <v>0.0548</v>
       </c>
       <c r="P22">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q22">
-        <v>1128</v>
+        <v>1742</v>
       </c>
       <c r="R22">
-        <v>62.028</v>
+        <v>95.6752</v>
       </c>
       <c r="S22" t="s">
         <v>33</v>
@@ -6571,7 +6595,7 @@
         <v>32</v>
       </c>
       <c r="G25">
-        <v>1.07257792</v>
+        <v>1.07216533</v>
       </c>
       <c r="H25">
         <v>1.075</v>
@@ -6586,25 +6610,25 @@
         <v>1.08</v>
       </c>
       <c r="L25">
-        <v>1.06</v>
+        <v>1.065</v>
       </c>
       <c r="M25">
-        <v>-1.85</v>
+        <v>-1.39</v>
       </c>
       <c r="N25">
         <v>1.06</v>
       </c>
       <c r="O25">
-        <v>1.08</v>
+        <v>1.075</v>
       </c>
       <c r="P25">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q25">
-        <v>1893</v>
+        <v>2002</v>
       </c>
       <c r="R25">
-        <v>2030.39</v>
+        <v>2146.475</v>
       </c>
       <c r="S25" t="s">
         <v>43</v>
@@ -6695,7 +6719,7 @@
         <v>32</v>
       </c>
       <c r="G27">
-        <v>0.64593359</v>
+        <v>0.64594582</v>
       </c>
       <c r="H27">
         <v>0.647</v>
@@ -6710,25 +6734,22 @@
         <v>0.646</v>
       </c>
       <c r="L27">
-        <v>0.647</v>
-      </c>
-      <c r="M27">
-        <v>0.15</v>
+        <v>0.646</v>
       </c>
       <c r="N27">
         <v>0.646</v>
       </c>
       <c r="O27">
-        <v>0.647</v>
+        <v>0.646</v>
       </c>
       <c r="P27">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="Q27">
-        <v>115420</v>
+        <v>129893</v>
       </c>
       <c r="R27">
-        <v>74553.655</v>
+        <v>83903.841</v>
       </c>
       <c r="S27" t="s">
         <v>43</v>
@@ -6757,7 +6778,7 @@
         <v>32</v>
       </c>
       <c r="G28">
-        <v>9.02400323</v>
+        <v>9.01369341</v>
       </c>
       <c r="H28">
         <v>9.05</v>
@@ -6778,19 +6799,19 @@
         <v>-0.44</v>
       </c>
       <c r="N28">
-        <v>9.0</v>
+        <v>9.01</v>
       </c>
       <c r="O28">
         <v>9.01</v>
       </c>
       <c r="P28">
-        <v>282</v>
+        <v>404</v>
       </c>
       <c r="Q28">
-        <v>6190</v>
+        <v>10979</v>
       </c>
       <c r="R28">
-        <v>55858.58</v>
+        <v>98961.34</v>
       </c>
       <c r="S28" t="s">
         <v>43</v>
@@ -6860,7 +6881,7 @@
         <v>32</v>
       </c>
       <c r="G30">
-        <v>1.21106577</v>
+        <v>1.21113757</v>
       </c>
       <c r="H30">
         <v>1.208</v>
@@ -6884,16 +6905,16 @@
         <v>1.21</v>
       </c>
       <c r="O30">
-        <v>1.212</v>
+        <v>1.214</v>
       </c>
       <c r="P30">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="Q30">
-        <v>17683</v>
+        <v>18696</v>
       </c>
       <c r="R30">
-        <v>21415.276</v>
+        <v>22643.428</v>
       </c>
       <c r="S30" t="s">
         <v>26</v>
@@ -6922,7 +6943,7 @@
         <v>32</v>
       </c>
       <c r="G31">
-        <v>10.88387609</v>
+        <v>10.87583128</v>
       </c>
       <c r="H31">
         <v>10.85</v>
@@ -6946,13 +6967,13 @@
         <v>10.85</v>
       </c>
       <c r="P31">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="Q31">
-        <v>1259</v>
+        <v>1624</v>
       </c>
       <c r="R31">
-        <v>13702.8</v>
+        <v>17662.35</v>
       </c>
       <c r="S31" t="s">
         <v>111</v>
@@ -7067,7 +7088,7 @@
         <v>38</v>
       </c>
       <c r="G2">
-        <v>1.26965818</v>
+        <v>1.26891858</v>
       </c>
       <c r="H2">
         <v>1.27</v>
@@ -7076,31 +7097,31 @@
         <v>1.305</v>
       </c>
       <c r="J2">
-        <v>1.26</v>
+        <v>1.255</v>
       </c>
       <c r="K2">
         <v>1.275</v>
       </c>
       <c r="L2">
-        <v>1.27</v>
+        <v>1.255</v>
       </c>
       <c r="M2">
-        <v>-0.39</v>
+        <v>-1.57</v>
       </c>
       <c r="N2">
         <v>1.26</v>
       </c>
       <c r="O2">
-        <v>1.275</v>
+        <v>1.27</v>
       </c>
       <c r="P2">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="Q2">
-        <v>746</v>
+        <v>786</v>
       </c>
       <c r="R2">
-        <v>947.165</v>
+        <v>997.37</v>
       </c>
       <c r="S2" t="s">
         <v>33</v>
@@ -7129,7 +7150,7 @@
         <v>32</v>
       </c>
       <c r="G3">
-        <v>1.6709477</v>
+        <v>1.67140037</v>
       </c>
       <c r="H3">
         <v>1.65</v>
@@ -7150,19 +7171,19 @@
         <v>2.13</v>
       </c>
       <c r="N3">
-        <v>1.67</v>
+        <v>1.675</v>
       </c>
       <c r="O3">
         <v>1.675</v>
       </c>
       <c r="P3">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="Q3">
-        <v>19236</v>
+        <v>20259</v>
       </c>
       <c r="R3">
-        <v>32142.35</v>
+        <v>33860.9</v>
       </c>
       <c r="S3" t="s">
         <v>63</v>
@@ -7191,7 +7212,7 @@
         <v>25</v>
       </c>
       <c r="G4">
-        <v>6.75136986</v>
+        <v>6.75202703</v>
       </c>
       <c r="H4">
         <v>6.75</v>
@@ -7206,10 +7227,10 @@
         <v>6.7</v>
       </c>
       <c r="L4">
-        <v>6.75</v>
+        <v>6.8</v>
       </c>
       <c r="M4">
-        <v>0.75</v>
+        <v>1.49</v>
       </c>
       <c r="N4">
         <v>6.7</v>
@@ -7218,13 +7239,13 @@
         <v>6.8</v>
       </c>
       <c r="P4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q4">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="R4">
-        <v>1971.4</v>
+        <v>1998.6</v>
       </c>
       <c r="S4" t="s">
         <v>33</v>
@@ -7341,7 +7362,7 @@
         <v>32</v>
       </c>
       <c r="G7">
-        <v>9.83996115</v>
+        <v>9.85407324</v>
       </c>
       <c r="H7">
         <v>9.74</v>
@@ -7356,25 +7377,25 @@
         <v>9.72</v>
       </c>
       <c r="L7">
-        <v>9.88</v>
+        <v>9.9</v>
       </c>
       <c r="M7">
-        <v>1.65</v>
+        <v>1.85</v>
       </c>
       <c r="N7">
-        <v>9.86</v>
+        <v>9.92</v>
       </c>
       <c r="O7">
-        <v>9.88</v>
+        <v>9.96</v>
       </c>
       <c r="P7">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="Q7">
-        <v>2574</v>
+        <v>3550</v>
       </c>
       <c r="R7">
-        <v>25328.06</v>
+        <v>34981.96</v>
       </c>
       <c r="S7" t="s">
         <v>63</v>
@@ -7465,13 +7486,13 @@
         <v>25</v>
       </c>
       <c r="G9">
-        <v>12.1</v>
+        <v>12.10882353</v>
       </c>
       <c r="H9">
         <v>12.1</v>
       </c>
       <c r="I9">
-        <v>12.1</v>
+        <v>12.2</v>
       </c>
       <c r="J9">
         <v>12.1</v>
@@ -7480,7 +7501,10 @@
         <v>12.1</v>
       </c>
       <c r="L9">
-        <v>12.1</v>
+        <v>12.2</v>
+      </c>
+      <c r="M9">
+        <v>0.83</v>
       </c>
       <c r="N9">
         <v>12.1</v>
@@ -7489,13 +7513,13 @@
         <v>12.2</v>
       </c>
       <c r="P9">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q9">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="R9">
-        <v>1125.3</v>
+        <v>1235.1</v>
       </c>
       <c r="S9" t="s">
         <v>33</v>
@@ -7551,13 +7575,13 @@
         <v>10.45</v>
       </c>
       <c r="P10">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q10">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="R10">
-        <v>20.8</v>
+        <v>1060.8</v>
       </c>
       <c r="S10" t="s">
         <v>43</v>
@@ -7586,7 +7610,7 @@
         <v>38</v>
       </c>
       <c r="G11">
-        <v>0.33</v>
+        <v>0.30092308</v>
       </c>
       <c r="H11">
         <v>0.33</v>
@@ -7595,31 +7619,31 @@
         <v>0.33</v>
       </c>
       <c r="J11">
-        <v>0.33</v>
+        <v>0.294</v>
       </c>
       <c r="K11">
         <v>0.32</v>
       </c>
       <c r="L11">
-        <v>0.33</v>
+        <v>0.294</v>
       </c>
       <c r="M11">
-        <v>3.13</v>
+        <v>-8.13</v>
       </c>
       <c r="N11">
         <v>0.292</v>
       </c>
       <c r="O11">
-        <v>0.33</v>
+        <v>0.328</v>
       </c>
       <c r="P11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q11">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="R11">
-        <v>1.65</v>
+        <v>7.824</v>
       </c>
       <c r="S11" t="s">
         <v>26</v>
@@ -7648,7 +7672,7 @@
         <v>32</v>
       </c>
       <c r="G12">
-        <v>16.43611111</v>
+        <v>16.44252137</v>
       </c>
       <c r="H12">
         <v>16.5</v>
@@ -7663,25 +7687,25 @@
         <v>16.6</v>
       </c>
       <c r="L12">
-        <v>16.4</v>
+        <v>16.5</v>
       </c>
       <c r="M12">
-        <v>-1.2</v>
+        <v>-0.6</v>
       </c>
       <c r="N12">
-        <v>16.4</v>
+        <v>16.5</v>
       </c>
       <c r="O12">
-        <v>16.45</v>
+        <v>16.5</v>
       </c>
       <c r="P12">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="Q12">
-        <v>54</v>
+        <v>234</v>
       </c>
       <c r="R12">
-        <v>887.55</v>
+        <v>3847.55</v>
       </c>
       <c r="S12" t="s">
         <v>154</v>
@@ -7751,7 +7775,7 @@
         <v>25</v>
       </c>
       <c r="G14">
-        <v>4.41469127</v>
+        <v>4.41570577</v>
       </c>
       <c r="H14">
         <v>4.43</v>
@@ -7775,13 +7799,13 @@
         <v>4.43</v>
       </c>
       <c r="P14">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q14">
-        <v>1409</v>
+        <v>1509</v>
       </c>
       <c r="R14">
-        <v>6220.3</v>
+        <v>6663.3</v>
       </c>
       <c r="S14" t="s">
         <v>43</v>
@@ -8020,7 +8044,7 @@
         <v>32</v>
       </c>
       <c r="G4">
-        <v>3.84457939</v>
+        <v>3.84450608</v>
       </c>
       <c r="H4">
         <v>3.85</v>
@@ -8035,22 +8059,25 @@
         <v>3.85</v>
       </c>
       <c r="L4">
-        <v>3.85</v>
+        <v>3.84</v>
+      </c>
+      <c r="M4">
+        <v>-0.26</v>
       </c>
       <c r="N4">
         <v>3.84</v>
       </c>
       <c r="O4">
-        <v>3.85</v>
+        <v>3.84</v>
       </c>
       <c r="P4">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="Q4">
-        <v>4125</v>
+        <v>4525</v>
       </c>
       <c r="R4">
-        <v>15858.89</v>
+        <v>17396.39</v>
       </c>
       <c r="S4" t="s">
         <v>43</v>
@@ -8079,7 +8106,7 @@
         <v>38</v>
       </c>
       <c r="G5">
-        <v>0.08512414</v>
+        <v>0.08509359</v>
       </c>
       <c r="H5">
         <v>0.085</v>
@@ -8088,31 +8115,28 @@
         <v>0.0878</v>
       </c>
       <c r="J5">
-        <v>0.0842</v>
+        <v>0.0838</v>
       </c>
       <c r="K5">
         <v>0.085</v>
       </c>
       <c r="L5">
-        <v>0.0842</v>
-      </c>
-      <c r="M5">
-        <v>-0.94</v>
+        <v>0.085</v>
       </c>
       <c r="N5">
-        <v>0.0842</v>
+        <v>0.085</v>
       </c>
       <c r="O5">
         <v>0.085</v>
       </c>
       <c r="P5">
-        <v>349</v>
+        <v>370</v>
       </c>
       <c r="Q5">
-        <v>53623</v>
+        <v>55380</v>
       </c>
       <c r="R5">
-        <v>4564.612</v>
+        <v>4712.483</v>
       </c>
       <c r="S5" t="s">
         <v>33</v>
@@ -8182,7 +8206,7 @@
         <v>25</v>
       </c>
       <c r="G7">
-        <v>11.04245283</v>
+        <v>11.02836879</v>
       </c>
       <c r="H7">
         <v>11.2</v>
@@ -8191,31 +8215,31 @@
         <v>11.3</v>
       </c>
       <c r="J7">
-        <v>11.0</v>
+        <v>10.9</v>
       </c>
       <c r="K7">
         <v>11.2</v>
       </c>
       <c r="L7">
-        <v>11.0</v>
+        <v>10.9</v>
       </c>
       <c r="M7">
-        <v>-1.79</v>
+        <v>-2.68</v>
       </c>
       <c r="N7">
         <v>10.9</v>
       </c>
       <c r="O7">
-        <v>11.0</v>
+        <v>10.9</v>
       </c>
       <c r="P7">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="Q7">
-        <v>106</v>
+        <v>141</v>
       </c>
       <c r="R7">
-        <v>1170.5</v>
+        <v>1555.0</v>
       </c>
       <c r="S7" t="s">
         <v>26</v>
@@ -8244,7 +8268,7 @@
         <v>32</v>
       </c>
       <c r="G8">
-        <v>1.01965205</v>
+        <v>1.01976436</v>
       </c>
       <c r="H8">
         <v>1.02</v>
@@ -8268,13 +8292,13 @@
         <v>1.02</v>
       </c>
       <c r="P8">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="Q8">
-        <v>1049</v>
+        <v>1549</v>
       </c>
       <c r="R8">
-        <v>1069.615</v>
+        <v>1579.615</v>
       </c>
       <c r="S8" t="s">
         <v>97</v>
@@ -8303,7 +8327,7 @@
         <v>32</v>
       </c>
       <c r="G9">
-        <v>21.77170331</v>
+        <v>21.76905795</v>
       </c>
       <c r="H9">
         <v>21.85</v>
@@ -8330,13 +8354,13 @@
         <v>21.75</v>
       </c>
       <c r="P9">
-        <v>368</v>
+        <v>402</v>
       </c>
       <c r="Q9">
-        <v>22151</v>
+        <v>24659</v>
       </c>
       <c r="R9">
-        <v>482265.0</v>
+        <v>536803.2</v>
       </c>
       <c r="S9" t="s">
         <v>111</v>
@@ -8551,13 +8575,13 @@
         <v>27.0</v>
       </c>
       <c r="P13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q13">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="R13">
-        <v>2484.0</v>
+        <v>2511.0</v>
       </c>
       <c r="S13" t="s">
         <v>63</v>
@@ -8586,7 +8610,7 @@
         <v>32</v>
       </c>
       <c r="G14">
-        <v>0.48434724</v>
+        <v>0.48435317</v>
       </c>
       <c r="H14">
         <v>0.484</v>
@@ -8607,19 +8631,19 @@
         <v>0.21</v>
       </c>
       <c r="N14">
-        <v>0.484</v>
+        <v>0.485</v>
       </c>
       <c r="O14">
         <v>0.485</v>
       </c>
       <c r="P14">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="Q14">
-        <v>11557</v>
+        <v>11663</v>
       </c>
       <c r="R14">
-        <v>5597.601</v>
+        <v>5649.011</v>
       </c>
       <c r="S14" t="s">
         <v>26</v>
@@ -8648,7 +8672,7 @@
         <v>38</v>
       </c>
       <c r="G15">
-        <v>2.11112882</v>
+        <v>2.11162907</v>
       </c>
       <c r="H15">
         <v>2.1</v>
@@ -8672,16 +8696,16 @@
         <v>2.06</v>
       </c>
       <c r="O15">
-        <v>2.12</v>
+        <v>2.14</v>
       </c>
       <c r="P15">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q15">
-        <v>1506</v>
+        <v>1596</v>
       </c>
       <c r="R15">
-        <v>3179.36</v>
+        <v>3370.16</v>
       </c>
       <c r="S15" t="s">
         <v>111</v>
@@ -8710,7 +8734,7 @@
         <v>38</v>
       </c>
       <c r="G16">
-        <v>1.14065164</v>
+        <v>1.13956083</v>
       </c>
       <c r="H16">
         <v>1.14</v>
@@ -8719,13 +8743,16 @@
         <v>1.15</v>
       </c>
       <c r="J16">
-        <v>1.14</v>
+        <v>1.135</v>
       </c>
       <c r="K16">
         <v>1.14</v>
       </c>
       <c r="L16">
-        <v>1.14</v>
+        <v>1.135</v>
+      </c>
+      <c r="M16">
+        <v>-0.44</v>
       </c>
       <c r="N16">
         <v>1.135</v>
@@ -8734,13 +8761,13 @@
         <v>1.14</v>
       </c>
       <c r="P16">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q16">
-        <v>2839</v>
+        <v>3518</v>
       </c>
       <c r="R16">
-        <v>3238.31</v>
+        <v>4008.975</v>
       </c>
       <c r="S16" t="s">
         <v>111</v>
@@ -8834,7 +8861,7 @@
         <v>0.75</v>
       </c>
       <c r="O18">
-        <v>0.76</v>
+        <v>0.758</v>
       </c>
       <c r="P18">
         <v>9</v>
@@ -8872,7 +8899,7 @@
         <v>32</v>
       </c>
       <c r="G19">
-        <v>1.80693753</v>
+        <v>1.80693339</v>
       </c>
       <c r="H19">
         <v>1.81</v>
@@ -8887,22 +8914,25 @@
         <v>1.81</v>
       </c>
       <c r="L19">
-        <v>1.81</v>
+        <v>1.805</v>
+      </c>
+      <c r="M19">
+        <v>-0.28</v>
       </c>
       <c r="N19">
-        <v>1.805</v>
+        <v>1.8</v>
       </c>
       <c r="O19">
         <v>1.81</v>
       </c>
       <c r="P19">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="Q19">
-        <v>2449</v>
+        <v>2462</v>
       </c>
       <c r="R19">
-        <v>4425.19</v>
+        <v>4448.67</v>
       </c>
       <c r="S19" t="s">
         <v>33</v>
@@ -8931,7 +8961,7 @@
         <v>32</v>
       </c>
       <c r="G20">
-        <v>0.89654925</v>
+        <v>0.89632286</v>
       </c>
       <c r="H20">
         <v>0.9</v>
@@ -8940,31 +8970,31 @@
         <v>0.9</v>
       </c>
       <c r="J20">
-        <v>0.895</v>
+        <v>0.894</v>
       </c>
       <c r="K20">
         <v>0.9</v>
       </c>
       <c r="L20">
-        <v>0.896</v>
+        <v>0.894</v>
       </c>
       <c r="M20">
-        <v>-0.44</v>
+        <v>-0.67</v>
       </c>
       <c r="N20">
         <v>0.894</v>
       </c>
       <c r="O20">
-        <v>0.896</v>
+        <v>0.894</v>
       </c>
       <c r="P20">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="Q20">
-        <v>107255</v>
+        <v>122187</v>
       </c>
       <c r="R20">
-        <v>96159.39</v>
+        <v>109519.001</v>
       </c>
     </row>
     <row r="21" spans="1:20">
@@ -8987,7 +9017,7 @@
         <v>32</v>
       </c>
       <c r="G21">
-        <v>4.45593909</v>
+        <v>4.4731934</v>
       </c>
       <c r="H21">
         <v>4.54</v>
@@ -9002,7 +9032,10 @@
         <v>4.5</v>
       </c>
       <c r="L21">
-        <v>4.5</v>
+        <v>4.48</v>
+      </c>
+      <c r="M21">
+        <v>-0.44</v>
       </c>
       <c r="N21">
         <v>4.46</v>
@@ -9011,13 +9044,13 @@
         <v>4.52</v>
       </c>
       <c r="P21">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="Q21">
-        <v>788</v>
+        <v>2668</v>
       </c>
       <c r="R21">
-        <v>3511.28</v>
+        <v>11934.48</v>
       </c>
       <c r="S21" t="s">
         <v>33</v>
@@ -9046,7 +9079,7 @@
         <v>32</v>
       </c>
       <c r="G22">
-        <v>2.2314222</v>
+        <v>2.23209208</v>
       </c>
       <c r="H22">
         <v>2.23</v>
@@ -9073,13 +9106,13 @@
         <v>2.24</v>
       </c>
       <c r="P22">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="Q22">
-        <v>28934</v>
+        <v>31385</v>
       </c>
       <c r="R22">
-        <v>64563.97</v>
+        <v>70054.21</v>
       </c>
       <c r="S22" t="s">
         <v>154</v>
@@ -9108,7 +9141,7 @@
         <v>38</v>
       </c>
       <c r="G23">
-        <v>0.33606832</v>
+        <v>0.32764706</v>
       </c>
       <c r="H23">
         <v>0.34</v>
@@ -9117,31 +9150,31 @@
         <v>0.34</v>
       </c>
       <c r="J23">
-        <v>0.334</v>
+        <v>0.32</v>
       </c>
       <c r="K23">
         <v>0.34</v>
       </c>
       <c r="L23">
-        <v>0.334</v>
+        <v>0.32</v>
       </c>
       <c r="M23">
-        <v>-1.76</v>
+        <v>-5.88</v>
       </c>
       <c r="N23">
-        <v>0.334</v>
+        <v>0.32</v>
       </c>
       <c r="O23">
         <v>0.34</v>
       </c>
       <c r="P23">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="Q23">
-        <v>322</v>
+        <v>850</v>
       </c>
       <c r="R23">
-        <v>108.214</v>
+        <v>278.5</v>
       </c>
       <c r="S23" t="s">
         <v>43</v>
@@ -9170,7 +9203,7 @@
         <v>38</v>
       </c>
       <c r="G24">
-        <v>9.87631579</v>
+        <v>9.85</v>
       </c>
       <c r="H24">
         <v>9.85</v>
@@ -9179,13 +9212,16 @@
         <v>9.9</v>
       </c>
       <c r="J24">
-        <v>9.85</v>
+        <v>9.6</v>
       </c>
       <c r="K24">
         <v>9.9</v>
       </c>
       <c r="L24">
-        <v>9.9</v>
+        <v>9.6</v>
+      </c>
+      <c r="M24">
+        <v>-3.03</v>
       </c>
       <c r="N24">
         <v>9.6</v>
@@ -9194,13 +9230,13 @@
         <v>9.9</v>
       </c>
       <c r="P24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q24">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="R24">
-        <v>187.65</v>
+        <v>206.85</v>
       </c>
       <c r="S24" t="s">
         <v>43</v>
@@ -9229,7 +9265,7 @@
         <v>32</v>
       </c>
       <c r="G25">
-        <v>15.30085586</v>
+        <v>15.30082322</v>
       </c>
       <c r="H25">
         <v>15.3</v>
@@ -9256,13 +9292,13 @@
         <v>15.3</v>
       </c>
       <c r="P25">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="Q25">
-        <v>1110</v>
+        <v>1154</v>
       </c>
       <c r="R25">
-        <v>16983.95</v>
+        <v>17657.15</v>
       </c>
       <c r="S25" t="s">
         <v>33</v>
@@ -9291,13 +9327,13 @@
         <v>38</v>
       </c>
       <c r="G26">
-        <v>2.9433126</v>
+        <v>2.94375191</v>
       </c>
       <c r="H26">
         <v>2.94</v>
       </c>
       <c r="I26">
-        <v>2.96</v>
+        <v>2.98</v>
       </c>
       <c r="J26">
         <v>2.9</v>
@@ -9306,10 +9342,10 @@
         <v>2.94</v>
       </c>
       <c r="L26">
-        <v>2.96</v>
+        <v>2.98</v>
       </c>
       <c r="M26">
-        <v>0.68</v>
+        <v>1.36</v>
       </c>
       <c r="N26">
         <v>2.94</v>
@@ -9318,13 +9354,13 @@
         <v>2.98</v>
       </c>
       <c r="P26">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="Q26">
-        <v>1286</v>
+        <v>1306</v>
       </c>
       <c r="R26">
-        <v>3785.1</v>
+        <v>3844.54</v>
       </c>
       <c r="S26" t="s">
         <v>33</v>

</xml_diff>